<commit_message>
added the 2s fixtures
</commit_message>
<xml_diff>
--- a/in/MRFC-FIXTURES-2025-26.xlsx
+++ b/in/MRFC-FIXTURES-2025-26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickgreen/workspace/code/morleyrfc/morleyrfc-fixtures/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C39282-6672-A945-BAA2-80FFC7351FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574FDD0D-8722-804E-A602-E33F90232769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="760" windowWidth="21820" windowHeight="16440" tabRatio="482" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="146">
   <si>
     <t>Date</t>
   </si>
@@ -453,6 +453,33 @@
   </si>
   <si>
     <t>York</t>
+  </si>
+  <si>
+    <t>Huddersfield</t>
+  </si>
+  <si>
+    <t>Harrogate</t>
+  </si>
+  <si>
+    <t>Heath</t>
+  </si>
+  <si>
+    <t>Hunslet Wolves</t>
+  </si>
+  <si>
+    <t>Keighley</t>
+  </si>
+  <si>
+    <t>Cleckheaton</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Wath Upon Dearne</t>
   </si>
 </sst>
 </file>
@@ -1775,8 +1802,12 @@
         <v>31</v>
       </c>
       <c r="C8" s="93"/>
-      <c r="D8" s="65"/>
-      <c r="E8" s="56"/>
+      <c r="D8" s="65" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="56" t="s">
+        <v>143</v>
+      </c>
       <c r="F8" s="6"/>
       <c r="G8" s="36"/>
       <c r="H8" s="36"/>
@@ -1794,8 +1825,12 @@
         <v>132</v>
       </c>
       <c r="C9" s="93"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="57"/>
+      <c r="D9" s="65" t="s">
+        <v>138</v>
+      </c>
+      <c r="E9" s="57" t="s">
+        <v>144</v>
+      </c>
       <c r="F9" s="6"/>
       <c r="G9" s="36"/>
       <c r="H9" s="36"/>
@@ -1813,8 +1848,12 @@
         <v>133</v>
       </c>
       <c r="C10" s="93"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="56"/>
+      <c r="D10" s="64" t="s">
+        <v>145</v>
+      </c>
+      <c r="E10" s="56" t="s">
+        <v>143</v>
+      </c>
       <c r="F10" s="4"/>
       <c r="G10" s="36"/>
       <c r="H10" s="36"/>
@@ -1851,8 +1890,12 @@
         <v>11</v>
       </c>
       <c r="C12" s="93"/>
-      <c r="D12" s="64"/>
-      <c r="E12" s="58"/>
+      <c r="D12" s="64" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" s="58" t="s">
+        <v>143</v>
+      </c>
       <c r="F12" s="4"/>
       <c r="G12" s="40"/>
       <c r="H12" s="40"/>
@@ -1870,8 +1913,12 @@
         <v>32</v>
       </c>
       <c r="C13" s="93"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="59"/>
+      <c r="D13" s="66" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="59" t="s">
+        <v>143</v>
+      </c>
       <c r="F13" s="4"/>
       <c r="G13" s="36"/>
       <c r="H13" s="35"/>
@@ -1889,8 +1936,12 @@
         <v>129</v>
       </c>
       <c r="C14" s="93"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="59"/>
+      <c r="D14" s="66" t="s">
+        <v>129</v>
+      </c>
+      <c r="E14" s="59" t="s">
+        <v>144</v>
+      </c>
       <c r="F14" s="4"/>
       <c r="G14" s="40"/>
       <c r="H14" s="42"/>
@@ -1909,8 +1960,12 @@
         <v>30</v>
       </c>
       <c r="C15" s="93"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="57"/>
+      <c r="D15" s="64" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>144</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="40"/>
       <c r="H15" s="40"/>
@@ -1947,8 +2002,12 @@
         <v>33</v>
       </c>
       <c r="C17" s="93"/>
-      <c r="D17" s="64"/>
-      <c r="E17" s="56"/>
+      <c r="D17" s="64" t="s">
+        <v>141</v>
+      </c>
+      <c r="E17" s="56" t="s">
+        <v>143</v>
+      </c>
       <c r="F17" s="4"/>
       <c r="G17" s="41"/>
       <c r="H17" s="42"/>
@@ -1986,8 +2045,12 @@
         <v>130</v>
       </c>
       <c r="C19" s="93"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="61"/>
+      <c r="D19" s="64" t="s">
+        <v>142</v>
+      </c>
+      <c r="E19" s="61" t="s">
+        <v>143</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="40"/>
       <c r="H19" s="35"/>
@@ -2006,8 +2069,12 @@
         <v>12</v>
       </c>
       <c r="C20" s="93"/>
-      <c r="D20" s="64"/>
-      <c r="E20" s="57"/>
+      <c r="D20" s="64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="57" t="s">
+        <v>144</v>
+      </c>
       <c r="F20" s="4"/>
       <c r="G20" s="41"/>
       <c r="H20" s="42"/>
@@ -2026,8 +2093,12 @@
         <v>13</v>
       </c>
       <c r="C21" s="93"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="57"/>
+      <c r="D21" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="57" t="s">
+        <v>143</v>
+      </c>
       <c r="F21" s="6"/>
       <c r="G21" s="36"/>
       <c r="H21" s="35"/>
@@ -2045,8 +2116,12 @@
         <v>132</v>
       </c>
       <c r="C22" s="93"/>
-      <c r="D22" s="65"/>
-      <c r="E22" s="62"/>
+      <c r="D22" s="65" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22" s="62" t="s">
+        <v>144</v>
+      </c>
       <c r="F22" s="4"/>
       <c r="G22" s="36"/>
       <c r="H22" s="35"/>
@@ -2121,8 +2196,12 @@
         <v>11</v>
       </c>
       <c r="C26" s="93"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
+      <c r="D26" s="62" t="s">
+        <v>139</v>
+      </c>
+      <c r="E26" s="62" t="s">
+        <v>144</v>
+      </c>
       <c r="F26" s="52"/>
       <c r="G26" s="35"/>
       <c r="H26" s="39"/>
@@ -2140,8 +2219,12 @@
         <v>32</v>
       </c>
       <c r="C27" s="93"/>
-      <c r="D27" s="64"/>
-      <c r="E27" s="56"/>
+      <c r="D27" s="64" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="56" t="s">
+        <v>144</v>
+      </c>
       <c r="F27" s="4"/>
       <c r="G27" s="40"/>
       <c r="H27" s="34"/>
@@ -2178,8 +2261,12 @@
         <v>129</v>
       </c>
       <c r="C29" s="93"/>
-      <c r="D29" s="64"/>
-      <c r="E29" s="56"/>
+      <c r="D29" s="64" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="56" t="s">
+        <v>144</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="40"/>
       <c r="H29" s="34"/>
@@ -2197,8 +2284,12 @@
         <v>134</v>
       </c>
       <c r="C30" s="93"/>
-      <c r="D30" s="64"/>
-      <c r="E30" s="59"/>
+      <c r="D30" s="64" t="s">
+        <v>145</v>
+      </c>
+      <c r="E30" s="59" t="s">
+        <v>144</v>
+      </c>
       <c r="F30" s="5"/>
       <c r="G30" s="40"/>
       <c r="H30" s="34"/>
@@ -2216,8 +2307,12 @@
         <v>30</v>
       </c>
       <c r="C31" s="93"/>
-      <c r="D31" s="67"/>
-      <c r="E31" s="56"/>
+      <c r="D31" s="67" t="s">
+        <v>129</v>
+      </c>
+      <c r="E31" s="56" t="s">
+        <v>143</v>
+      </c>
       <c r="F31" s="4"/>
       <c r="G31" s="40"/>
       <c r="H31" s="34"/>
@@ -2235,8 +2330,12 @@
         <v>134</v>
       </c>
       <c r="C32" s="93"/>
-      <c r="D32" s="66"/>
-      <c r="E32" s="56"/>
+      <c r="D32" s="66" t="s">
+        <v>138</v>
+      </c>
+      <c r="E32" s="56" t="s">
+        <v>143</v>
+      </c>
       <c r="F32" s="5"/>
       <c r="G32" s="36"/>
       <c r="H32" s="38"/>
@@ -2274,8 +2373,12 @@
         <v>130</v>
       </c>
       <c r="C34" s="93"/>
-      <c r="D34" s="64"/>
-      <c r="E34" s="59"/>
+      <c r="D34" s="64" t="s">
+        <v>141</v>
+      </c>
+      <c r="E34" s="59" t="s">
+        <v>144</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="40"/>
       <c r="H34" s="34"/>
@@ -2312,8 +2415,12 @@
         <v>12</v>
       </c>
       <c r="C36" s="93"/>
-      <c r="D36" s="64"/>
-      <c r="E36" s="56"/>
+      <c r="D36" s="64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="56" t="s">
+        <v>143</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="40"/>
       <c r="H36" s="38"/>
@@ -2332,8 +2439,12 @@
         <v>13</v>
       </c>
       <c r="C37" s="93"/>
-      <c r="D37" s="66"/>
-      <c r="E37" s="56"/>
+      <c r="D37" s="66" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="56" t="s">
+        <v>144</v>
+      </c>
       <c r="F37" s="5"/>
       <c r="G37" s="40"/>
       <c r="H37" s="34"/>
@@ -2370,8 +2481,12 @@
         <v>31</v>
       </c>
       <c r="C39" s="93"/>
-      <c r="D39" s="66"/>
-      <c r="E39" s="59"/>
+      <c r="D39" s="66" t="s">
+        <v>140</v>
+      </c>
+      <c r="E39" s="59" t="s">
+        <v>143</v>
+      </c>
       <c r="F39" s="5"/>
       <c r="G39" s="41"/>
       <c r="H39" s="41"/>

</xml_diff>

<commit_message>
added yorkshire cup fixture
</commit_message>
<xml_diff>
--- a/in/MRFC-FIXTURES-2025-26.xlsx
+++ b/in/MRFC-FIXTURES-2025-26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickgreen/workspace/code/morleyrfc/morleyrfc-fixtures/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574FDD0D-8722-804E-A602-E33F90232769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520AB0EC-A126-BB4C-8E5E-C6323DBBF0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="760" windowWidth="21820" windowHeight="16440" tabRatio="482" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="149">
   <si>
     <t>Date</t>
   </si>
@@ -480,6 +480,15 @@
   </si>
   <si>
     <t>Wath Upon Dearne</t>
+  </si>
+  <si>
+    <t>Malton &amp; Norton (YC)</t>
+  </si>
+  <si>
+    <t>H*</t>
+  </si>
+  <si>
+    <t>A*</t>
   </si>
 </sst>
 </file>
@@ -1731,7 +1740,9 @@
       <c r="B4" s="88" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="91"/>
+      <c r="C4" s="91" t="s">
+        <v>144</v>
+      </c>
       <c r="D4" s="72"/>
       <c r="E4" s="73"/>
       <c r="F4" s="74"/>
@@ -1801,7 +1812,9 @@
       <c r="B8" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="93"/>
+      <c r="C8" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D8" s="65" t="s">
         <v>137</v>
       </c>
@@ -1824,7 +1837,9 @@
       <c r="B9" s="90" t="s">
         <v>132</v>
       </c>
-      <c r="C9" s="93"/>
+      <c r="C9" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D9" s="65" t="s">
         <v>138</v>
       </c>
@@ -1847,7 +1862,9 @@
       <c r="B10" s="90" t="s">
         <v>133</v>
       </c>
-      <c r="C10" s="93"/>
+      <c r="C10" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D10" s="64" t="s">
         <v>145</v>
       </c>
@@ -1868,9 +1885,11 @@
         <v>45927</v>
       </c>
       <c r="B11" s="90" t="s">
-        <v>134</v>
-      </c>
-      <c r="C11" s="93"/>
+        <v>146</v>
+      </c>
+      <c r="C11" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D11" s="64"/>
       <c r="E11" s="57"/>
       <c r="F11" s="4"/>
@@ -1889,7 +1908,9 @@
       <c r="B12" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="93"/>
+      <c r="C12" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D12" s="64" t="s">
         <v>139</v>
       </c>
@@ -1912,7 +1933,9 @@
       <c r="B13" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="93"/>
+      <c r="C13" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D13" s="66" t="s">
         <v>32</v>
       </c>
@@ -1935,7 +1958,9 @@
       <c r="B14" s="90" t="s">
         <v>129</v>
       </c>
-      <c r="C14" s="93"/>
+      <c r="C14" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D14" s="66" t="s">
         <v>129</v>
       </c>
@@ -1959,7 +1984,9 @@
       <c r="B15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="93"/>
+      <c r="C15" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D15" s="64" t="s">
         <v>140</v>
       </c>
@@ -2001,7 +2028,9 @@
       <c r="B17" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="93"/>
+      <c r="C17" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D17" s="64" t="s">
         <v>141</v>
       </c>
@@ -2044,7 +2073,9 @@
       <c r="B19" s="90" t="s">
         <v>130</v>
       </c>
-      <c r="C19" s="93"/>
+      <c r="C19" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D19" s="64" t="s">
         <v>142</v>
       </c>
@@ -2068,7 +2099,9 @@
       <c r="B20" s="90" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="93"/>
+      <c r="C20" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D20" s="64" t="s">
         <v>12</v>
       </c>
@@ -2092,7 +2125,9 @@
       <c r="B21" s="90" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="93"/>
+      <c r="C21" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D21" s="64" t="s">
         <v>13</v>
       </c>
@@ -2115,7 +2150,9 @@
       <c r="B22" s="90" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="93"/>
+      <c r="C22" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D22" s="65" t="s">
         <v>142</v>
       </c>
@@ -2138,7 +2175,9 @@
       <c r="B23" s="90" t="s">
         <v>133</v>
       </c>
-      <c r="C23" s="93"/>
+      <c r="C23" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D23" s="66"/>
       <c r="E23" s="63"/>
       <c r="F23" s="5"/>
@@ -2195,7 +2234,9 @@
       <c r="B26" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="93"/>
+      <c r="C26" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D26" s="62" t="s">
         <v>139</v>
       </c>
@@ -2218,7 +2259,9 @@
       <c r="B27" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="93"/>
+      <c r="C27" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D27" s="64" t="s">
         <v>137</v>
       </c>
@@ -2260,7 +2303,9 @@
       <c r="B29" s="90" t="s">
         <v>129</v>
       </c>
-      <c r="C29" s="93"/>
+      <c r="C29" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D29" s="64" t="s">
         <v>32</v>
       </c>
@@ -2306,7 +2351,9 @@
       <c r="B31" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="93"/>
+      <c r="C31" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D31" s="67" t="s">
         <v>129</v>
       </c>
@@ -2353,7 +2400,9 @@
       <c r="B33" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="93"/>
+      <c r="C33" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D33" s="64"/>
       <c r="E33" s="56"/>
       <c r="F33" s="4"/>
@@ -2372,7 +2421,9 @@
       <c r="B34" s="90" t="s">
         <v>130</v>
       </c>
-      <c r="C34" s="93"/>
+      <c r="C34" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D34" s="64" t="s">
         <v>141</v>
       </c>
@@ -2414,7 +2465,9 @@
       <c r="B36" s="90" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="93"/>
+      <c r="C36" s="93" t="s">
+        <v>147</v>
+      </c>
       <c r="D36" s="64" t="s">
         <v>12</v>
       </c>
@@ -2438,7 +2491,9 @@
       <c r="B37" s="90" t="s">
         <v>13</v>
       </c>
-      <c r="C37" s="93"/>
+      <c r="C37" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D37" s="66" t="s">
         <v>13</v>
       </c>
@@ -2480,7 +2535,9 @@
       <c r="B39" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="93"/>
+      <c r="C39" s="93" t="s">
+        <v>148</v>
+      </c>
       <c r="D39" s="66" t="s">
         <v>140</v>
       </c>

</xml_diff>

<commit_message>
fix: update to cavs comps
</commit_message>
<xml_diff>
--- a/in/MRFC-FIXTURES-2025-26.xlsx
+++ b/in/MRFC-FIXTURES-2025-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickgreen/workspace/code/morleyrfc/morleyrfc-fixtures/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520AB0EC-A126-BB4C-8E5E-C6323DBBF0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19318476-8DD3-5D41-87D2-486A980E997E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="760" windowWidth="21820" windowHeight="16440" tabRatio="482" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="148">
   <si>
     <t>Date</t>
   </si>
@@ -471,9 +471,6 @@
   </si>
   <si>
     <t>Cleckheaton</t>
-  </si>
-  <si>
-    <t>A</t>
   </si>
   <si>
     <t>H</t>
@@ -498,7 +495,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,13 +611,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1110,7 +1100,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1241,9 +1231,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1301,7 +1288,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1669,20 +1656,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="94" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="97"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
+      <c r="L1" s="96"/>
       <c r="N1"/>
       <c r="O1"/>
     </row>
@@ -1698,7 +1685,7 @@
       <c r="I2" s="54"/>
       <c r="J2" s="54"/>
       <c r="K2" s="54"/>
-      <c r="L2" s="71"/>
+      <c r="L2" s="70"/>
     </row>
     <row r="3" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1707,28 +1694,28 @@
       <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="77" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="79" t="s">
+      <c r="D3" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="78" t="s">
+      <c r="E3" s="77" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="80"/>
-      <c r="G3" s="81" t="s">
+      <c r="F3" s="79"/>
+      <c r="G3" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="82" t="s">
+      <c r="H3" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="83"/>
-      <c r="J3" s="84" t="s">
+      <c r="I3" s="82"/>
+      <c r="J3" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="84"/>
-      <c r="L3" s="85" t="s">
+      <c r="K3" s="83"/>
+      <c r="L3" s="84" t="s">
         <v>10</v>
       </c>
       <c r="O3"/>
@@ -1737,31 +1724,31 @@
       <c r="A4" s="3">
         <v>45883</v>
       </c>
-      <c r="B4" s="88" t="s">
+      <c r="B4" s="87" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="91" t="s">
-        <v>144</v>
-      </c>
-      <c r="D4" s="72"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
-      <c r="I4" s="75"/>
-      <c r="J4" s="76"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="77"/>
+      <c r="C4" s="90" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="71"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="74"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="74"/>
+      <c r="L4" s="76"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="68">
+      <c r="A5" s="67">
         <v>45890</v>
       </c>
-      <c r="B5" s="89" t="s">
+      <c r="B5" s="88" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="92"/>
-      <c r="D5" s="64"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="63"/>
       <c r="E5" s="55"/>
       <c r="F5" s="4"/>
       <c r="G5" s="34"/>
@@ -1772,14 +1759,14 @@
       <c r="L5" s="47"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="68">
+      <c r="A6" s="67">
         <v>45899</v>
       </c>
-      <c r="B6" s="89" t="s">
+      <c r="B6" s="88" t="s">
         <v>136</v>
       </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="64"/>
+      <c r="C6" s="91"/>
+      <c r="D6" s="63"/>
       <c r="E6" s="55"/>
       <c r="F6" s="4"/>
       <c r="G6" s="34"/>
@@ -1787,15 +1774,15 @@
       <c r="I6" s="34"/>
       <c r="J6" s="33"/>
       <c r="K6" s="34"/>
-      <c r="L6" s="86"/>
+      <c r="L6" s="85"/>
     </row>
     <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="69">
+      <c r="A7" s="68">
         <v>45536</v>
       </c>
-      <c r="B7" s="89"/>
-      <c r="C7" s="92"/>
-      <c r="D7" s="64"/>
+      <c r="B7" s="88"/>
+      <c r="C7" s="91"/>
+      <c r="D7" s="63"/>
       <c r="E7" s="55"/>
       <c r="F7" s="4"/>
       <c r="G7" s="34"/>
@@ -1806,20 +1793,20 @@
       <c r="L7" s="47"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="68">
+      <c r="A8" s="67">
         <v>45906</v>
       </c>
-      <c r="B8" s="90" t="s">
+      <c r="B8" s="89" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="93" t="s">
+      <c r="C8" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="64" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="92" t="s">
         <v>147</v>
-      </c>
-      <c r="D8" s="65" t="s">
-        <v>137</v>
-      </c>
-      <c r="E8" s="56" t="s">
-        <v>143</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="36"/>
@@ -1830,21 +1817,21 @@
       <c r="L8" s="48"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="68">
+      <c r="A9" s="67">
         <f>+A8+7</f>
         <v>45913</v>
       </c>
-      <c r="B9" s="90" t="s">
+      <c r="B9" s="89" t="s">
         <v>132</v>
       </c>
-      <c r="C9" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D9" s="65" t="s">
+      <c r="C9" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D9" s="64" t="s">
         <v>138</v>
       </c>
-      <c r="E9" s="57" t="s">
-        <v>144</v>
+      <c r="E9" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="36"/>
@@ -1855,21 +1842,21 @@
       <c r="L9" s="49"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="68">
+      <c r="A10" s="67">
         <f t="shared" ref="A10:A22" si="0">+A9+7</f>
         <v>45920</v>
       </c>
-      <c r="B10" s="90" t="s">
+      <c r="B10" s="89" t="s">
         <v>133</v>
       </c>
-      <c r="C10" s="93" t="s">
+      <c r="C10" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D10" s="63" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="92" t="s">
         <v>147</v>
-      </c>
-      <c r="D10" s="64" t="s">
-        <v>145</v>
-      </c>
-      <c r="E10" s="56" t="s">
-        <v>143</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="36"/>
@@ -1880,17 +1867,17 @@
       <c r="L10" s="50"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="68">
+      <c r="A11" s="67">
         <f t="shared" si="0"/>
         <v>45927</v>
       </c>
-      <c r="B11" s="90" t="s">
+      <c r="B11" s="89" t="s">
+        <v>145</v>
+      </c>
+      <c r="C11" s="92" t="s">
         <v>146</v>
       </c>
-      <c r="C11" s="93" t="s">
-        <v>147</v>
-      </c>
-      <c r="D11" s="64"/>
+      <c r="D11" s="63"/>
       <c r="E11" s="57"/>
       <c r="F11" s="4"/>
       <c r="G11" s="40"/>
@@ -1901,21 +1888,21 @@
       <c r="L11" s="50"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="68">
+      <c r="A12" s="67">
         <f t="shared" si="0"/>
         <v>45934</v>
       </c>
-      <c r="B12" s="90" t="s">
+      <c r="B12" s="89" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D12" s="64" t="s">
+      <c r="C12" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D12" s="63" t="s">
         <v>139</v>
       </c>
-      <c r="E12" s="58" t="s">
-        <v>143</v>
+      <c r="E12" s="92" t="s">
+        <v>147</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="40"/>
@@ -1926,21 +1913,21 @@
       <c r="L12" s="50"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="68">
+      <c r="A13" s="67">
         <f t="shared" si="0"/>
         <v>45941</v>
       </c>
-      <c r="B13" s="90" t="s">
+      <c r="B13" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="93" t="s">
+      <c r="C13" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D13" s="65" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="92" t="s">
         <v>147</v>
-      </c>
-      <c r="D13" s="66" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="59" t="s">
-        <v>143</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="36"/>
@@ -1951,21 +1938,21 @@
       <c r="L13" s="50"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="68">
+      <c r="A14" s="67">
         <f t="shared" si="0"/>
         <v>45948</v>
       </c>
-      <c r="B14" s="90" t="s">
+      <c r="B14" s="89" t="s">
         <v>129</v>
       </c>
-      <c r="C14" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D14" s="66" t="s">
+      <c r="C14" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D14" s="65" t="s">
         <v>129</v>
       </c>
-      <c r="E14" s="59" t="s">
-        <v>144</v>
+      <c r="E14" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="40"/>
@@ -1977,21 +1964,21 @@
       <c r="O14"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="68">
+      <c r="A15" s="67">
         <f t="shared" si="0"/>
         <v>45955</v>
       </c>
-      <c r="B15" s="90" t="s">
+      <c r="B15" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="93" t="s">
-        <v>147</v>
-      </c>
-      <c r="D15" s="64" t="s">
+      <c r="C15" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="63" t="s">
         <v>140</v>
       </c>
-      <c r="E15" s="57" t="s">
-        <v>144</v>
+      <c r="E15" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="40"/>
@@ -2002,15 +1989,15 @@
       <c r="L15" s="50"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="68">
+      <c r="A16" s="67">
         <f t="shared" si="0"/>
         <v>45962</v>
       </c>
-      <c r="B16" s="90" t="s">
+      <c r="B16" s="89" t="s">
         <v>134</v>
       </c>
-      <c r="C16" s="93"/>
-      <c r="D16" s="64"/>
+      <c r="C16" s="92"/>
+      <c r="D16" s="63"/>
       <c r="E16" s="60"/>
       <c r="F16" s="4"/>
       <c r="G16" s="40"/>
@@ -2021,21 +2008,21 @@
       <c r="L16" s="50"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="68">
+      <c r="A17" s="67">
         <f t="shared" si="0"/>
         <v>45969</v>
       </c>
-      <c r="B17" s="90" t="s">
+      <c r="B17" s="89" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D17" s="64" t="s">
+      <c r="C17" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="E17" s="56" t="s">
-        <v>143</v>
+      <c r="E17" s="92" t="s">
+        <v>147</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="41"/>
@@ -2046,15 +2033,15 @@
       <c r="L17" s="50"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="68">
+      <c r="A18" s="67">
         <f t="shared" si="0"/>
         <v>45976</v>
       </c>
-      <c r="B18" s="87" t="s">
+      <c r="B18" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="93"/>
-      <c r="D18" s="64"/>
+      <c r="C18" s="92"/>
+      <c r="D18" s="63"/>
       <c r="E18" s="57"/>
       <c r="F18" s="4"/>
       <c r="G18" s="41"/>
@@ -2066,21 +2053,21 @@
       <c r="N18" s="8"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="68">
+      <c r="A19" s="67">
         <f t="shared" si="0"/>
         <v>45983</v>
       </c>
-      <c r="B19" s="90" t="s">
+      <c r="B19" s="89" t="s">
         <v>130</v>
       </c>
-      <c r="C19" s="93" t="s">
+      <c r="C19" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D19" s="63" t="s">
+        <v>142</v>
+      </c>
+      <c r="E19" s="92" t="s">
         <v>147</v>
-      </c>
-      <c r="D19" s="64" t="s">
-        <v>142</v>
-      </c>
-      <c r="E19" s="61" t="s">
-        <v>143</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="40"/>
@@ -2092,21 +2079,21 @@
       <c r="N19" s="8"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="68">
+      <c r="A20" s="67">
         <f t="shared" si="0"/>
         <v>45990</v>
       </c>
-      <c r="B20" s="90" t="s">
+      <c r="B20" s="89" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D20" s="64" t="s">
+      <c r="C20" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="57" t="s">
-        <v>144</v>
+      <c r="E20" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="41"/>
@@ -2118,21 +2105,21 @@
       <c r="N20" s="9"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A21" s="68">
+      <c r="A21" s="67">
         <f t="shared" si="0"/>
         <v>45997</v>
       </c>
-      <c r="B21" s="90" t="s">
+      <c r="B21" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="93" t="s">
+      <c r="C21" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="63" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="92" t="s">
         <v>147</v>
-      </c>
-      <c r="D21" s="64" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="57" t="s">
-        <v>143</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="36"/>
@@ -2143,21 +2130,21 @@
       <c r="L21" s="50"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A22" s="68">
+      <c r="A22" s="67">
         <f t="shared" si="0"/>
         <v>46004</v>
       </c>
-      <c r="B22" s="90" t="s">
+      <c r="B22" s="89" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="93" t="s">
-        <v>147</v>
-      </c>
-      <c r="D22" s="65" t="s">
+      <c r="C22" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D22" s="64" t="s">
         <v>142</v>
       </c>
-      <c r="E22" s="62" t="s">
-        <v>144</v>
+      <c r="E22" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="36"/>
@@ -2168,18 +2155,18 @@
       <c r="L22" s="50"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A23" s="68">
+      <c r="A23" s="67">
         <f>+A22+7</f>
         <v>46011</v>
       </c>
-      <c r="B23" s="90" t="s">
+      <c r="B23" s="89" t="s">
         <v>133</v>
       </c>
-      <c r="C23" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D23" s="66"/>
-      <c r="E23" s="63"/>
+      <c r="C23" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D23" s="65"/>
+      <c r="E23" s="62"/>
       <c r="F23" s="5"/>
       <c r="G23" s="41"/>
       <c r="H23" s="41"/>
@@ -2189,15 +2176,15 @@
       <c r="L23" s="50"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A24" s="70">
+      <c r="A24" s="69">
         <f>+A23+7</f>
         <v>46018</v>
       </c>
-      <c r="B24" s="90" t="s">
+      <c r="B24" s="89" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="93"/>
-      <c r="D24" s="66"/>
+      <c r="C24" s="92"/>
+      <c r="D24" s="65"/>
       <c r="E24" s="59"/>
       <c r="F24" s="5"/>
       <c r="G24" s="41"/>
@@ -2208,15 +2195,15 @@
       <c r="L24" s="50"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A25" s="68">
+      <c r="A25" s="67">
         <f t="shared" ref="A25:A37" si="1">+A24+7</f>
         <v>46025</v>
       </c>
-      <c r="B25" s="87" t="s">
+      <c r="B25" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="C25" s="93"/>
-      <c r="D25" s="66"/>
+      <c r="C25" s="92"/>
+      <c r="D25" s="65"/>
       <c r="E25" s="59"/>
       <c r="F25" s="5"/>
       <c r="G25" s="41"/>
@@ -2227,21 +2214,21 @@
       <c r="L25" s="50"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A26" s="68">
+      <c r="A26" s="67">
         <f t="shared" si="1"/>
         <v>46032</v>
       </c>
-      <c r="B26" s="90" t="s">
+      <c r="B26" s="89" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="93" t="s">
-        <v>147</v>
-      </c>
-      <c r="D26" s="62" t="s">
+      <c r="C26" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D26" s="61" t="s">
         <v>139</v>
       </c>
-      <c r="E26" s="62" t="s">
-        <v>144</v>
+      <c r="E26" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F26" s="52"/>
       <c r="G26" s="35"/>
@@ -2252,21 +2239,21 @@
       <c r="L26" s="50"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A27" s="68">
+      <c r="A27" s="67">
         <f t="shared" si="1"/>
         <v>46039</v>
       </c>
-      <c r="B27" s="90" t="s">
+      <c r="B27" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D27" s="64" t="s">
+      <c r="C27" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="63" t="s">
         <v>137</v>
       </c>
-      <c r="E27" s="56" t="s">
-        <v>144</v>
+      <c r="E27" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="40"/>
@@ -2277,15 +2264,15 @@
       <c r="L27" s="50"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A28" s="68">
+      <c r="A28" s="67">
         <f t="shared" si="1"/>
         <v>46046</v>
       </c>
-      <c r="B28" s="87" t="s">
+      <c r="B28" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="C28" s="93"/>
-      <c r="D28" s="64"/>
+      <c r="C28" s="92"/>
+      <c r="D28" s="63"/>
       <c r="E28" s="56"/>
       <c r="F28" s="4"/>
       <c r="G28" s="40"/>
@@ -2296,21 +2283,21 @@
       <c r="L28" s="50"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A29" s="68">
+      <c r="A29" s="67">
         <f t="shared" si="1"/>
         <v>46053</v>
       </c>
-      <c r="B29" s="90" t="s">
+      <c r="B29" s="89" t="s">
         <v>129</v>
       </c>
-      <c r="C29" s="93" t="s">
-        <v>147</v>
-      </c>
-      <c r="D29" s="64" t="s">
+      <c r="C29" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D29" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="E29" s="56" t="s">
-        <v>144</v>
+      <c r="E29" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="40"/>
@@ -2321,19 +2308,19 @@
       <c r="L29" s="50"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A30" s="68">
+      <c r="A30" s="67">
         <f t="shared" si="1"/>
         <v>46060</v>
       </c>
-      <c r="B30" s="90" t="s">
+      <c r="B30" s="89" t="s">
         <v>134</v>
       </c>
-      <c r="C30" s="93"/>
-      <c r="D30" s="64" t="s">
-        <v>145</v>
-      </c>
-      <c r="E30" s="59" t="s">
+      <c r="C30" s="92"/>
+      <c r="D30" s="63" t="s">
         <v>144</v>
+      </c>
+      <c r="E30" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="40"/>
@@ -2344,21 +2331,21 @@
       <c r="L30" s="50"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A31" s="68">
+      <c r="A31" s="67">
         <f t="shared" si="1"/>
         <v>46067</v>
       </c>
-      <c r="B31" s="90" t="s">
+      <c r="B31" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D31" s="67" t="s">
+      <c r="C31" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D31" s="66" t="s">
         <v>129</v>
       </c>
-      <c r="E31" s="56" t="s">
-        <v>143</v>
+      <c r="E31" s="92" t="s">
+        <v>147</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="40"/>
@@ -2369,19 +2356,19 @@
       <c r="L31" s="50"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A32" s="68">
+      <c r="A32" s="67">
         <f t="shared" si="1"/>
         <v>46074</v>
       </c>
-      <c r="B32" s="87" t="s">
+      <c r="B32" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="C32" s="93"/>
-      <c r="D32" s="66" t="s">
+      <c r="C32" s="92"/>
+      <c r="D32" s="65" t="s">
         <v>138</v>
       </c>
-      <c r="E32" s="56" t="s">
-        <v>143</v>
+      <c r="E32" s="92" t="s">
+        <v>147</v>
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="36"/>
@@ -2393,17 +2380,17 @@
       <c r="O32"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A33" s="68">
+      <c r="A33" s="67">
         <f t="shared" si="1"/>
         <v>46081</v>
       </c>
-      <c r="B33" s="90" t="s">
+      <c r="B33" s="89" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="93" t="s">
-        <v>147</v>
-      </c>
-      <c r="D33" s="64"/>
+      <c r="C33" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D33" s="63"/>
       <c r="E33" s="56"/>
       <c r="F33" s="4"/>
       <c r="G33" s="40"/>
@@ -2414,21 +2401,21 @@
       <c r="L33" s="50"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A34" s="68">
+      <c r="A34" s="67">
         <f t="shared" si="1"/>
         <v>46088</v>
       </c>
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>130</v>
       </c>
-      <c r="C34" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D34" s="64" t="s">
+      <c r="C34" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D34" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="E34" s="59" t="s">
-        <v>144</v>
+      <c r="E34" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="40"/>
@@ -2439,15 +2426,15 @@
       <c r="L34" s="50"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A35" s="68">
+      <c r="A35" s="67">
         <f t="shared" si="1"/>
         <v>46095</v>
       </c>
-      <c r="B35" s="87" t="s">
+      <c r="B35" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="C35" s="93"/>
-      <c r="D35" s="66"/>
+      <c r="C35" s="92"/>
+      <c r="D35" s="65"/>
       <c r="E35" s="58"/>
       <c r="F35" s="5"/>
       <c r="G35" s="41"/>
@@ -2458,21 +2445,21 @@
       <c r="L35" s="50"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A36" s="68">
+      <c r="A36" s="67">
         <f t="shared" si="1"/>
         <v>46102</v>
       </c>
-      <c r="B36" s="90" t="s">
+      <c r="B36" s="89" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="93" t="s">
+      <c r="C36" s="92" t="s">
+        <v>146</v>
+      </c>
+      <c r="D36" s="63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="92" t="s">
         <v>147</v>
-      </c>
-      <c r="D36" s="64" t="s">
-        <v>12</v>
-      </c>
-      <c r="E36" s="56" t="s">
-        <v>143</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="40"/>
@@ -2484,21 +2471,21 @@
       <c r="N36" s="11"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A37" s="68">
+      <c r="A37" s="67">
         <f t="shared" si="1"/>
         <v>46109</v>
       </c>
-      <c r="B37" s="90" t="s">
+      <c r="B37" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="C37" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D37" s="66" t="s">
+      <c r="C37" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D37" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="E37" s="56" t="s">
-        <v>144</v>
+      <c r="E37" s="92" t="s">
+        <v>146</v>
       </c>
       <c r="F37" s="5"/>
       <c r="G37" s="40"/>
@@ -2509,15 +2496,15 @@
       <c r="L37" s="50"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A38" s="68">
+      <c r="A38" s="67">
         <f>+A37+7</f>
         <v>46116</v>
       </c>
-      <c r="B38" s="87" t="s">
+      <c r="B38" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="93"/>
-      <c r="D38" s="66"/>
+      <c r="C38" s="92"/>
+      <c r="D38" s="65"/>
       <c r="E38" s="56"/>
       <c r="F38" s="5"/>
       <c r="G38" s="36"/>
@@ -2528,21 +2515,21 @@
       <c r="L38" s="50"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A39" s="70">
+      <c r="A39" s="69">
         <f>+A38+7</f>
         <v>46123</v>
       </c>
-      <c r="B39" s="90" t="s">
+      <c r="B39" s="89" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="93" t="s">
-        <v>148</v>
-      </c>
-      <c r="D39" s="66" t="s">
+      <c r="C39" s="92" t="s">
+        <v>147</v>
+      </c>
+      <c r="D39" s="65" t="s">
         <v>140</v>
       </c>
-      <c r="E39" s="59" t="s">
-        <v>143</v>
+      <c r="E39" s="92" t="s">
+        <v>147</v>
       </c>
       <c r="F39" s="5"/>
       <c r="G39" s="41"/>
@@ -2553,15 +2540,15 @@
       <c r="L39" s="50"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A40" s="68">
+      <c r="A40" s="67">
         <f t="shared" ref="A40:A43" si="2">+A39+7</f>
         <v>46130</v>
       </c>
-      <c r="B40" s="90" t="s">
+      <c r="B40" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="C40" s="93"/>
-      <c r="D40" s="64"/>
+      <c r="C40" s="92"/>
+      <c r="D40" s="63"/>
       <c r="E40" s="56"/>
       <c r="F40" s="6"/>
       <c r="G40" s="40"/>
@@ -2572,15 +2559,15 @@
       <c r="L40" s="50"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A41" s="68">
+      <c r="A41" s="67">
         <f t="shared" si="2"/>
         <v>46137</v>
       </c>
-      <c r="B41" s="90" t="s">
+      <c r="B41" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="C41" s="93"/>
-      <c r="D41" s="66"/>
+      <c r="C41" s="92"/>
+      <c r="D41" s="65"/>
       <c r="E41" s="56"/>
       <c r="F41" s="4"/>
       <c r="G41" s="40"/>
@@ -2591,15 +2578,15 @@
       <c r="L41" s="50"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A42" s="68">
+      <c r="A42" s="67">
         <f t="shared" si="2"/>
         <v>46144</v>
       </c>
-      <c r="B42" s="90" t="s">
+      <c r="B42" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="C42" s="93"/>
-      <c r="D42" s="66"/>
+      <c r="C42" s="92"/>
+      <c r="D42" s="65"/>
       <c r="E42" s="56"/>
       <c r="F42" s="4"/>
       <c r="G42" s="40"/>
@@ -2610,15 +2597,15 @@
       <c r="L42" s="50"/>
     </row>
     <row r="43" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="68">
+      <c r="A43" s="67">
         <f t="shared" si="2"/>
         <v>46151</v>
       </c>
-      <c r="B43" s="90" t="s">
+      <c r="B43" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="C43" s="94"/>
-      <c r="D43" s="66"/>
+      <c r="C43" s="93"/>
+      <c r="D43" s="65"/>
       <c r="E43" s="56"/>
       <c r="F43" s="4"/>
       <c r="G43" s="40"/>

</xml_diff>